<commit_message>
feat(invoice): 更新发票模板文件 CHY.xlsx 和 GHZX.xlsx
</commit_message>
<xml_diff>
--- a/assests/invoice_template/CHY.xlsx
+++ b/assests/invoice_template/CHY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30720" windowHeight="13380"/>
+    <workbookView windowWidth="30720" windowHeight="13500"/>
   </bookViews>
   <sheets>
     <sheet name="开票申请单（测绘院） (3)" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
     <t>申请部门：</t>
   </si>
   <si>
-    <t>生产经营管理科</t>
+    <t>生产经营管理部</t>
   </si>
   <si>
     <t>申请日期：</t>
@@ -1910,14 +1910,14 @@
       <c r="AL7" s="20"/>
       <c r="AM7" s="20"/>
       <c r="AN7" s="20"/>
-      <c r="AO7" s="20"/>
-      <c r="AP7" s="20"/>
-      <c r="AQ7" s="20"/>
-      <c r="AR7" s="20"/>
-      <c r="AS7" s="20"/>
-      <c r="AT7" s="20"/>
-      <c r="AU7" s="20"/>
-      <c r="AV7" s="20"/>
+      <c r="AO7" s="33"/>
+      <c r="AP7" s="33"/>
+      <c r="AQ7" s="33"/>
+      <c r="AR7" s="33"/>
+      <c r="AS7" s="33"/>
+      <c r="AT7" s="33"/>
+      <c r="AU7" s="33"/>
+      <c r="AV7" s="33"/>
     </row>
     <row r="8" ht="37.5" customHeight="1" spans="1:48">
       <c r="A8" s="13"/>
@@ -1937,28 +1937,28 @@
       <c r="K8" s="20"/>
       <c r="L8" s="20"/>
       <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20"/>
-      <c r="Q8" s="20"/>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20"/>
-      <c r="T8" s="20"/>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20"/>
-      <c r="W8" s="20"/>
-      <c r="X8" s="20"/>
-      <c r="Y8" s="20"/>
-      <c r="Z8" s="20"/>
-      <c r="AA8" s="20"/>
-      <c r="AB8" s="20"/>
-      <c r="AC8" s="20"/>
-      <c r="AD8" s="20"/>
-      <c r="AE8" s="20"/>
-      <c r="AF8" s="20"/>
-      <c r="AG8" s="20"/>
-      <c r="AH8" s="20"/>
-      <c r="AI8" s="20"/>
+      <c r="N8" s="33"/>
+      <c r="O8" s="33"/>
+      <c r="P8" s="33"/>
+      <c r="Q8" s="33"/>
+      <c r="R8" s="33"/>
+      <c r="S8" s="33"/>
+      <c r="T8" s="33"/>
+      <c r="U8" s="33"/>
+      <c r="V8" s="33"/>
+      <c r="W8" s="33"/>
+      <c r="X8" s="33"/>
+      <c r="Y8" s="33"/>
+      <c r="Z8" s="33"/>
+      <c r="AA8" s="33"/>
+      <c r="AB8" s="33"/>
+      <c r="AC8" s="33"/>
+      <c r="AD8" s="33"/>
+      <c r="AE8" s="33"/>
+      <c r="AF8" s="33"/>
+      <c r="AG8" s="33"/>
+      <c r="AH8" s="33"/>
+      <c r="AI8" s="33"/>
       <c r="AJ8" s="20" t="s">
         <v>25</v>
       </c>
@@ -1966,14 +1966,14 @@
       <c r="AL8" s="20"/>
       <c r="AM8" s="20"/>
       <c r="AN8" s="20"/>
-      <c r="AO8" s="20"/>
-      <c r="AP8" s="20"/>
-      <c r="AQ8" s="20"/>
-      <c r="AR8" s="20"/>
-      <c r="AS8" s="20"/>
-      <c r="AT8" s="20"/>
-      <c r="AU8" s="20"/>
-      <c r="AV8" s="20"/>
+      <c r="AO8" s="33"/>
+      <c r="AP8" s="33"/>
+      <c r="AQ8" s="33"/>
+      <c r="AR8" s="33"/>
+      <c r="AS8" s="33"/>
+      <c r="AT8" s="33"/>
+      <c r="AU8" s="33"/>
+      <c r="AV8" s="33"/>
     </row>
     <row r="9" ht="37.5" customHeight="1" spans="1:48">
       <c r="A9" s="13"/>
@@ -2026,14 +2026,14 @@
       <c r="AL9" s="25"/>
       <c r="AM9" s="25"/>
       <c r="AN9" s="26"/>
-      <c r="AO9" s="24"/>
-      <c r="AP9" s="25"/>
-      <c r="AQ9" s="25"/>
-      <c r="AR9" s="25"/>
-      <c r="AS9" s="25"/>
-      <c r="AT9" s="25"/>
-      <c r="AU9" s="25"/>
-      <c r="AV9" s="26"/>
+      <c r="AO9" s="21"/>
+      <c r="AP9" s="22"/>
+      <c r="AQ9" s="22"/>
+      <c r="AR9" s="22"/>
+      <c r="AS9" s="22"/>
+      <c r="AT9" s="22"/>
+      <c r="AU9" s="22"/>
+      <c r="AV9" s="23"/>
     </row>
     <row r="10" ht="37.5" customHeight="1" spans="1:48">
       <c r="A10" s="4"/>
@@ -2053,28 +2053,28 @@
       <c r="K10" s="20"/>
       <c r="L10" s="20"/>
       <c r="M10" s="20"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="25"/>
-      <c r="P10" s="25"/>
-      <c r="Q10" s="25"/>
-      <c r="R10" s="25"/>
-      <c r="S10" s="25"/>
-      <c r="T10" s="25"/>
-      <c r="U10" s="25"/>
-      <c r="V10" s="25"/>
-      <c r="W10" s="25"/>
-      <c r="X10" s="25"/>
-      <c r="Y10" s="25"/>
-      <c r="Z10" s="25"/>
-      <c r="AA10" s="25"/>
-      <c r="AB10" s="25"/>
-      <c r="AC10" s="25"/>
-      <c r="AD10" s="25"/>
-      <c r="AE10" s="25"/>
-      <c r="AF10" s="25"/>
-      <c r="AG10" s="25"/>
-      <c r="AH10" s="25"/>
-      <c r="AI10" s="26"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22"/>
+      <c r="R10" s="22"/>
+      <c r="S10" s="22"/>
+      <c r="T10" s="22"/>
+      <c r="U10" s="22"/>
+      <c r="V10" s="22"/>
+      <c r="W10" s="22"/>
+      <c r="X10" s="22"/>
+      <c r="Y10" s="22"/>
+      <c r="Z10" s="22"/>
+      <c r="AA10" s="22"/>
+      <c r="AB10" s="22"/>
+      <c r="AC10" s="22"/>
+      <c r="AD10" s="22"/>
+      <c r="AE10" s="22"/>
+      <c r="AF10" s="22"/>
+      <c r="AG10" s="22"/>
+      <c r="AH10" s="22"/>
+      <c r="AI10" s="23"/>
       <c r="AJ10" s="20" t="s">
         <v>33</v>
       </c>
@@ -2082,14 +2082,14 @@
       <c r="AL10" s="20"/>
       <c r="AM10" s="20"/>
       <c r="AN10" s="20"/>
-      <c r="AO10" s="24"/>
-      <c r="AP10" s="25"/>
-      <c r="AQ10" s="25"/>
-      <c r="AR10" s="25"/>
-      <c r="AS10" s="25"/>
-      <c r="AT10" s="25"/>
-      <c r="AU10" s="25"/>
-      <c r="AV10" s="26"/>
+      <c r="AO10" s="21"/>
+      <c r="AP10" s="22"/>
+      <c r="AQ10" s="22"/>
+      <c r="AR10" s="22"/>
+      <c r="AS10" s="22"/>
+      <c r="AT10" s="22"/>
+      <c r="AU10" s="22"/>
+      <c r="AV10" s="23"/>
     </row>
     <row r="11" ht="37.5" customHeight="1" spans="1:48">
       <c r="A11" s="4"/>
@@ -2107,28 +2107,28 @@
       <c r="K11" s="20"/>
       <c r="L11" s="20"/>
       <c r="M11" s="20"/>
-      <c r="N11" s="24"/>
-      <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="25"/>
-      <c r="R11" s="25"/>
-      <c r="S11" s="25"/>
-      <c r="T11" s="25"/>
-      <c r="U11" s="25"/>
-      <c r="V11" s="25"/>
-      <c r="W11" s="25"/>
-      <c r="X11" s="25"/>
-      <c r="Y11" s="25"/>
-      <c r="Z11" s="25"/>
-      <c r="AA11" s="25"/>
-      <c r="AB11" s="25"/>
-      <c r="AC11" s="25"/>
-      <c r="AD11" s="25"/>
-      <c r="AE11" s="25"/>
-      <c r="AF11" s="25"/>
-      <c r="AG11" s="25"/>
-      <c r="AH11" s="25"/>
-      <c r="AI11" s="26"/>
+      <c r="N11" s="21"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="22"/>
+      <c r="Q11" s="22"/>
+      <c r="R11" s="22"/>
+      <c r="S11" s="22"/>
+      <c r="T11" s="22"/>
+      <c r="U11" s="22"/>
+      <c r="V11" s="22"/>
+      <c r="W11" s="22"/>
+      <c r="X11" s="22"/>
+      <c r="Y11" s="22"/>
+      <c r="Z11" s="22"/>
+      <c r="AA11" s="22"/>
+      <c r="AB11" s="22"/>
+      <c r="AC11" s="22"/>
+      <c r="AD11" s="22"/>
+      <c r="AE11" s="22"/>
+      <c r="AF11" s="22"/>
+      <c r="AG11" s="22"/>
+      <c r="AH11" s="22"/>
+      <c r="AI11" s="23"/>
       <c r="AJ11" s="20" t="s">
         <v>35</v>
       </c>
@@ -2136,14 +2136,14 @@
       <c r="AL11" s="20"/>
       <c r="AM11" s="20"/>
       <c r="AN11" s="20"/>
-      <c r="AO11" s="24"/>
-      <c r="AP11" s="25"/>
-      <c r="AQ11" s="25"/>
-      <c r="AR11" s="25"/>
-      <c r="AS11" s="25"/>
-      <c r="AT11" s="25"/>
-      <c r="AU11" s="25"/>
-      <c r="AV11" s="26"/>
+      <c r="AO11" s="21"/>
+      <c r="AP11" s="22"/>
+      <c r="AQ11" s="22"/>
+      <c r="AR11" s="22"/>
+      <c r="AS11" s="22"/>
+      <c r="AT11" s="22"/>
+      <c r="AU11" s="22"/>
+      <c r="AV11" s="23"/>
     </row>
     <row r="12" ht="37.5" customHeight="1" spans="1:48">
       <c r="A12" s="4"/>
@@ -2161,28 +2161,28 @@
       <c r="K12" s="20"/>
       <c r="L12" s="20"/>
       <c r="M12" s="20"/>
-      <c r="N12" s="24"/>
-      <c r="O12" s="25"/>
-      <c r="P12" s="25"/>
-      <c r="Q12" s="25"/>
-      <c r="R12" s="25"/>
-      <c r="S12" s="25"/>
-      <c r="T12" s="25"/>
-      <c r="U12" s="25"/>
-      <c r="V12" s="25"/>
-      <c r="W12" s="25"/>
-      <c r="X12" s="25"/>
-      <c r="Y12" s="25"/>
-      <c r="Z12" s="25"/>
-      <c r="AA12" s="25"/>
-      <c r="AB12" s="25"/>
-      <c r="AC12" s="25"/>
-      <c r="AD12" s="25"/>
-      <c r="AE12" s="25"/>
-      <c r="AF12" s="25"/>
-      <c r="AG12" s="25"/>
-      <c r="AH12" s="25"/>
-      <c r="AI12" s="26"/>
+      <c r="N12" s="21"/>
+      <c r="O12" s="22"/>
+      <c r="P12" s="22"/>
+      <c r="Q12" s="22"/>
+      <c r="R12" s="22"/>
+      <c r="S12" s="22"/>
+      <c r="T12" s="22"/>
+      <c r="U12" s="22"/>
+      <c r="V12" s="22"/>
+      <c r="W12" s="22"/>
+      <c r="X12" s="22"/>
+      <c r="Y12" s="22"/>
+      <c r="Z12" s="22"/>
+      <c r="AA12" s="22"/>
+      <c r="AB12" s="22"/>
+      <c r="AC12" s="22"/>
+      <c r="AD12" s="22"/>
+      <c r="AE12" s="22"/>
+      <c r="AF12" s="22"/>
+      <c r="AG12" s="22"/>
+      <c r="AH12" s="22"/>
+      <c r="AI12" s="23"/>
       <c r="AJ12" s="20" t="s">
         <v>37</v>
       </c>
@@ -2190,14 +2190,14 @@
       <c r="AL12" s="20"/>
       <c r="AM12" s="20"/>
       <c r="AN12" s="20"/>
-      <c r="AO12" s="24"/>
-      <c r="AP12" s="25"/>
-      <c r="AQ12" s="25"/>
-      <c r="AR12" s="25"/>
-      <c r="AS12" s="25"/>
-      <c r="AT12" s="25"/>
-      <c r="AU12" s="25"/>
-      <c r="AV12" s="26"/>
+      <c r="AO12" s="21"/>
+      <c r="AP12" s="22"/>
+      <c r="AQ12" s="22"/>
+      <c r="AR12" s="22"/>
+      <c r="AS12" s="22"/>
+      <c r="AT12" s="22"/>
+      <c r="AU12" s="22"/>
+      <c r="AV12" s="23"/>
     </row>
     <row r="13" ht="37.5" customHeight="1" spans="1:48">
       <c r="A13" s="13"/>

</xml_diff>